<commit_message>
OficinaIA: metadatos en biblioteca + boton slash en chat
</commit_message>
<xml_diff>
--- a/excel_interno.xlsx
+++ b/excel_interno.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASEGURADOS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z175"/>
+  <dimension ref="A1:Z180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11804,11 +11804,7 @@
       <c r="Z174" t="inlineStr"/>
     </row>
     <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>31 de agosto dar de baja brandan</t>
-        </is>
-      </c>
+      <c r="A175" t="inlineStr"/>
       <c r="B175" t="inlineStr"/>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr"/>
@@ -11835,6 +11831,174 @@
       <c r="Y175" t="inlineStr"/>
       <c r="Z175" t="inlineStr"/>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr"/>
+      <c r="B176" t="inlineStr"/>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr"/>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
+      <c r="P176" t="inlineStr"/>
+      <c r="Q176" t="inlineStr"/>
+      <c r="R176" t="inlineStr"/>
+      <c r="S176" t="inlineStr"/>
+      <c r="T176" t="inlineStr"/>
+      <c r="U176" t="inlineStr"/>
+      <c r="V176" t="inlineStr"/>
+      <c r="W176" t="inlineStr"/>
+      <c r="X176" t="inlineStr"/>
+      <c r="Y176" t="inlineStr"/>
+      <c r="Z176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr"/>
+      <c r="B177" t="inlineStr"/>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr"/>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
+      <c r="P177" t="inlineStr"/>
+      <c r="Q177" t="inlineStr"/>
+      <c r="R177" t="inlineStr"/>
+      <c r="S177" t="inlineStr"/>
+      <c r="T177" t="inlineStr"/>
+      <c r="U177" t="inlineStr"/>
+      <c r="V177" t="inlineStr"/>
+      <c r="W177" t="inlineStr"/>
+      <c r="X177" t="inlineStr"/>
+      <c r="Y177" t="inlineStr"/>
+      <c r="Z177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr"/>
+      <c r="B178" t="inlineStr"/>
+      <c r="C178" t="inlineStr"/>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr"/>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
+      <c r="P178" t="inlineStr"/>
+      <c r="Q178" t="inlineStr"/>
+      <c r="R178" t="inlineStr"/>
+      <c r="S178" t="inlineStr"/>
+      <c r="T178" t="inlineStr"/>
+      <c r="U178" t="inlineStr"/>
+      <c r="V178" t="inlineStr"/>
+      <c r="W178" t="inlineStr"/>
+      <c r="X178" t="inlineStr"/>
+      <c r="Y178" t="inlineStr"/>
+      <c r="Z178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>ramiro alejandro herrera</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>1141492756</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>brava nevada 125</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>a189zhp</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>cuponera</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr"/>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
+      <c r="P179" t="inlineStr"/>
+      <c r="Q179" t="inlineStr"/>
+      <c r="R179" t="inlineStr"/>
+      <c r="S179" t="inlineStr"/>
+      <c r="T179" t="inlineStr"/>
+      <c r="U179" t="inlineStr"/>
+      <c r="V179" t="inlineStr"/>
+      <c r="W179" t="inlineStr"/>
+      <c r="X179" t="inlineStr"/>
+      <c r="Y179" t="inlineStr"/>
+      <c r="Z179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr"/>
+      <c r="B180" t="inlineStr"/>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr"/>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
+      <c r="P180" t="inlineStr"/>
+      <c r="Q180" t="inlineStr"/>
+      <c r="R180" t="inlineStr"/>
+      <c r="S180" t="inlineStr"/>
+      <c r="T180" t="inlineStr"/>
+      <c r="U180" t="inlineStr"/>
+      <c r="V180" t="inlineStr"/>
+      <c r="W180" t="inlineStr"/>
+      <c r="X180" t="inlineStr"/>
+      <c r="Y180" t="inlineStr"/>
+      <c r="Z180" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizacion de codigo y plantillas
</commit_message>
<xml_diff>
--- a/excel_interno.xlsx
+++ b/excel_interno.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z180"/>
+  <dimension ref="A1:Z186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -11918,30 +11918,14 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ramiro alejandro herrera</t>
-        </is>
-      </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>1141492756</t>
-        </is>
-      </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>brava nevada 125</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
-        <is>
-          <t>a189zhp</t>
-        </is>
-      </c>
+          <t>ramiro alejandroherrera</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr"/>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="inlineStr"/>
       <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr">
-        <is>
-          <t>atm</t>
-        </is>
-      </c>
+      <c r="F179" t="inlineStr"/>
       <c r="G179" t="inlineStr">
         <is>
           <t>cuponera</t>
@@ -11972,11 +11956,7 @@
       <c r="B180" t="inlineStr"/>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>si</t>
-        </is>
-      </c>
+      <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr"/>
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr"/>
@@ -11999,6 +11979,322 @@
       <c r="Y180" t="inlineStr"/>
       <c r="Z180" t="inlineStr"/>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>ramiro herrera</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>1141492756</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>brava nevada 125</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>a189zhp</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>cuponera</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>1865</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>passegurosyriesgos@gmail.com</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr"/>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
+      <c r="P181" t="inlineStr"/>
+      <c r="Q181" t="inlineStr"/>
+      <c r="R181" t="inlineStr"/>
+      <c r="S181" t="inlineStr"/>
+      <c r="T181" t="inlineStr"/>
+      <c r="U181" t="inlineStr"/>
+      <c r="V181" t="inlineStr"/>
+      <c r="W181" t="inlineStr"/>
+      <c r="X181" t="inlineStr"/>
+      <c r="Y181" t="inlineStr"/>
+      <c r="Z181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>ramiro herrera</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>1141492756</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>brava nevada 125</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>a189zhp</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>cuponera</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>1865</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>pas.segurosyriesgos@gmail.com</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
+      <c r="P182" t="inlineStr"/>
+      <c r="Q182" t="inlineStr"/>
+      <c r="R182" t="inlineStr"/>
+      <c r="S182" t="inlineStr"/>
+      <c r="T182" t="inlineStr"/>
+      <c r="U182" t="inlineStr"/>
+      <c r="V182" t="inlineStr"/>
+      <c r="W182" t="inlineStr"/>
+      <c r="X182" t="inlineStr"/>
+      <c r="Y182" t="inlineStr"/>
+      <c r="Z182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>pepito</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>676767</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>latercera</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr"/>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>1764</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr"/>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
+      <c r="P183" t="inlineStr"/>
+      <c r="Q183" t="inlineStr"/>
+      <c r="R183" t="inlineStr"/>
+      <c r="S183" t="inlineStr"/>
+      <c r="T183" t="inlineStr"/>
+      <c r="U183" t="inlineStr"/>
+      <c r="V183" t="inlineStr"/>
+      <c r="W183" t="inlineStr"/>
+      <c r="X183" t="inlineStr"/>
+      <c r="Y183" t="inlineStr"/>
+      <c r="Z183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>TRANSPORTE ALEJO SRL</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>58813260</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>FLOTA COMPLETA (34 UNIDADES)</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>La Segunda</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr"/>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr"/>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr"/>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
+      <c r="P184" t="inlineStr"/>
+      <c r="Q184" t="inlineStr"/>
+      <c r="R184" t="inlineStr"/>
+      <c r="S184" t="inlineStr"/>
+      <c r="T184" t="inlineStr"/>
+      <c r="U184" t="inlineStr"/>
+      <c r="V184" t="inlineStr"/>
+      <c r="W184" t="inlineStr"/>
+      <c r="X184" t="inlineStr"/>
+      <c r="Y184" t="inlineStr"/>
+      <c r="Z184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>TRANSPORTE ALEJO SRL</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>58813260</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>FIAT STRADA 1.3 FIRE FLY FREEDOM CS 2025</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>AH638CX</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>La Segunda</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr"/>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr"/>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr"/>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
+      <c r="P185" t="inlineStr"/>
+      <c r="Q185" t="inlineStr"/>
+      <c r="R185" t="inlineStr"/>
+      <c r="S185" t="inlineStr"/>
+      <c r="T185" t="inlineStr"/>
+      <c r="U185" t="inlineStr"/>
+      <c r="V185" t="inlineStr"/>
+      <c r="W185" t="inlineStr"/>
+      <c r="X185" t="inlineStr"/>
+      <c r="Y185" t="inlineStr"/>
+      <c r="Z185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>ramiro herrera</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>1141492756</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>brava nevada 125</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>a189zhp</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>atm</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>cuponera</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>1865</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr"/>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
+      <c r="P186" t="inlineStr"/>
+      <c r="Q186" t="inlineStr"/>
+      <c r="R186" t="inlineStr"/>
+      <c r="S186" t="inlineStr"/>
+      <c r="T186" t="inlineStr"/>
+      <c r="U186" t="inlineStr"/>
+      <c r="V186" t="inlineStr"/>
+      <c r="W186" t="inlineStr"/>
+      <c r="X186" t="inlineStr"/>
+      <c r="Y186" t="inlineStr"/>
+      <c r="Z186" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>